<commit_message>
Updated pre-selection scoring model and prepared phase 2 criteria
</commit_message>
<xml_diff>
--- a/output/preselection_full_table.xlsx
+++ b/output/preselection_full_table.xlsx
@@ -483,7 +483,7 @@
         <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>2.6</v>
+        <v>2.649999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -511,63 +511,63 @@
         <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>29280</v>
+        <v>66420</v>
       </c>
       <c r="D4" t="n">
-        <v>71.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>66420</v>
+        <v>29280</v>
       </c>
       <c r="D5" t="n">
-        <v>84.90000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>2.2</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="6">
@@ -623,7 +623,7 @@
         <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>1.8</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="8">
@@ -651,7 +651,7 @@
         <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>1.6</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1.2</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="10">
@@ -735,7 +735,7 @@
         <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.6499999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -763,7 +763,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Refined pre-selection scoring logic and updated ranking outputs
</commit_message>
<xml_diff>
--- a/output/preselection_full_table.xlsx
+++ b/output/preselection_full_table.xlsx
@@ -461,57 +461,57 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10.6</v>
+        <v>48.8</v>
       </c>
       <c r="C2" t="n">
-        <v>52600</v>
+        <v>32590</v>
       </c>
       <c r="D2" t="n">
-        <v>87.3</v>
+        <v>74.5</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>2.649999999999999</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48.8</v>
+        <v>10.6</v>
       </c>
       <c r="C3" t="n">
-        <v>32590</v>
+        <v>52600</v>
       </c>
       <c r="D3" t="n">
-        <v>74.5</v>
+        <v>87.3</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>2.35</v>
+        <v>2.649999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -530,7 +530,7 @@
         <v>84.90000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -539,7 +539,7 @@
         <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>2.3</v>
+        <v>2.649999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -564,10 +564,10 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>2.05</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="6">
@@ -592,10 +592,10 @@
         <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="7">
@@ -617,13 +617,13 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>1.95</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="8">
@@ -645,116 +645,116 @@
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>1.65</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9.9</v>
+        <v>10.7</v>
       </c>
       <c r="C9" t="n">
-        <v>22560</v>
+        <v>26700</v>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>53.9</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>1.05</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.7</v>
+        <v>2.9</v>
       </c>
       <c r="C10" t="n">
-        <v>26700</v>
+        <v>27150</v>
       </c>
       <c r="D10" t="n">
-        <v>53.9</v>
+        <v>56.7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.9</v>
+        <v>5.4</v>
       </c>
       <c r="C11" t="n">
-        <v>27150</v>
+        <v>24000</v>
       </c>
       <c r="D11" t="n">
-        <v>56.7</v>
+        <v>60.6</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6499999999999999</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5.4</v>
+        <v>9.9</v>
       </c>
       <c r="C12" t="n">
-        <v>24000</v>
+        <v>22560</v>
       </c>
       <c r="D12" t="n">
-        <v>60.6</v>
+        <v>55</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -763,7 +763,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.35</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="13">
@@ -782,16 +782,16 @@
         <v>52.5</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>